<commit_message>
feat: integracao dos novos cenarios de 2024 e 2025
- Adicionados os novos CSVs dividindo Papis Peritos e Nao Peritos
- Atualizacao do csv_dump.json para suportar mapeamento correto de alteracoes de nomes
- Novas sessoes visuais no modo 4 para historico de mudancas de nomes
- Inclusao do status badge de cenario ativo no modo 5
- Resolucao de bugs com dicionario do json no modo comparativo
</commit_message>
<xml_diff>
--- a/Tabela_Conversao_Cargos.xlsx
+++ b/Tabela_Conversao_Cargos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maiap\OneDrive\Desktop\Desenvolvimento\Estudo_Atribuicoes_PCSP_2024\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maiap\OneDrive\Desktop\Desenvolvimento\Estudo_Atribuicoes_PCSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{587950E9-A331-4B98-AC72-68FE5C95CF7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC88D42-B96D-4AF9-8E4B-1212FC85E867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{BDD19391-5856-444F-A0AF-5F8BE44242C9}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{BDD19391-5856-444F-A0AF-5F8BE44242C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="46">
   <si>
     <t>Delegado de Polícia</t>
   </si>
@@ -117,6 +117,66 @@
   </si>
   <si>
     <t>Reestruturação 2024</t>
+  </si>
+  <si>
+    <t>Perito Oficial Criminal</t>
+  </si>
+  <si>
+    <t>Analista de Identificação Policial</t>
+  </si>
+  <si>
+    <t>Oficial de Perícia Criminal</t>
+  </si>
+  <si>
+    <t>Reestruturação Reunião 1 2025</t>
+  </si>
+  <si>
+    <t>Reestruturação Reunião 2 2025</t>
+  </si>
+  <si>
+    <t>Oficial Investigador de Polícia - Especialista Cartorário</t>
+  </si>
+  <si>
+    <t>Oficial Investigador de Polícia - Especialista Investigativo</t>
+  </si>
+  <si>
+    <t>Perito Oficial Criminal - Especialista Perícia Criminalística</t>
+  </si>
+  <si>
+    <t>Perito Oficial Criminal - Especialista Técnico Medicina Legal</t>
+  </si>
+  <si>
+    <t>Oficial de Perícia Criminal - Especialista Perícia Criminalística</t>
+  </si>
+  <si>
+    <t>Oficial de Perícia Criminal - Especialista Técnico Medicina Legal</t>
+  </si>
+  <si>
+    <t>Analista de Polícia Judiciária</t>
+  </si>
+  <si>
+    <t>Decreto 47788 / 1967</t>
+  </si>
+  <si>
+    <t>Pesquisador Datiloscópico</t>
+  </si>
+  <si>
+    <t>Datiloscopista</t>
+  </si>
+  <si>
+    <t>Radiotelegrafista</t>
+  </si>
+  <si>
+    <t>Motorista</t>
+  </si>
+  <si>
+    <t>Guarda de Presídio</t>
+  </si>
+  <si>
+    <t>Auxiliar de Autópsia</t>
+  </si>
+  <si>
+    <t>NÃO ENCONTRADO</t>
   </si>
 </sst>
 </file>
@@ -194,10 +254,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -517,15 +573,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7CA06EA-7EEC-4748-A6C4-DD62A4A55B38}">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="91.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="57.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="29.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
@@ -541,8 +599,17 @@
       <c r="E1" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -558,8 +625,17 @@
       <c r="E2" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -575,8 +651,17 @@
       <c r="E3" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -592,8 +677,17 @@
       <c r="E4" s="2" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -609,8 +703,17 @@
       <c r="E5" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -626,8 +729,17 @@
       <c r="E6" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -643,8 +755,17 @@
       <c r="E7" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -660,8 +781,17 @@
       <c r="E8" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -677,8 +807,17 @@
       <c r="E9" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -694,8 +833,17 @@
       <c r="E10" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -711,8 +859,17 @@
       <c r="E11" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -728,8 +885,17 @@
       <c r="E12" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -745,8 +911,17 @@
       <c r="E13" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -762,8 +937,17 @@
       <c r="E14" s="2" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -778,6 +962,15 @@
       </c>
       <c r="E15" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add assignment catalog view and update supporting data files
</commit_message>
<xml_diff>
--- a/Tabela_Conversao_Cargos.xlsx
+++ b/Tabela_Conversao_Cargos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maiap\OneDrive\Desktop\Desenvolvimento\Estudo_Atribuicoes_PCSP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BC88D42-B96D-4AF9-8E4B-1212FC85E867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FAA1D4F-9515-40A6-8985-7BAB7C5A6BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{BDD19391-5856-444F-A0AF-5F8BE44242C9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="48">
   <si>
     <t>Delegado de Polícia</t>
   </si>
@@ -176,7 +176,13 @@
     <t>Auxiliar de Autópsia</t>
   </si>
   <si>
-    <t>NÃO ENCONTRADO</t>
+    <t>Fiscal de Diversões Públicas</t>
+  </si>
+  <si>
+    <t>Fotógrafo</t>
+  </si>
+  <si>
+    <t>Desenhista</t>
   </si>
 </sst>
 </file>
@@ -658,7 +664,7 @@
         <v>15</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -684,7 +690,7 @@
         <v>15</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>2</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -892,7 +898,7 @@
         <v>28</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -918,7 +924,7 @@
         <v>28</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -970,7 +976,7 @@
         <v>28</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>